<commit_message>
Add Excel formatting and report preview
</commit_message>
<xml_diff>
--- a/invoice_batch_report.xlsx
+++ b/invoice_batch_report.xlsx
@@ -9,14 +9,18 @@
   <sheets>
     <sheet name="Invoice Report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Invoice Report'!$A$1:$L$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -29,12 +33,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,9 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,9 +438,9 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -527,13 +539,13 @@
           <t>September 16, 2026</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="2" t="n">
         <v>850</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="2" t="n">
         <v>918</v>
       </c>
       <c r="J2" t="inlineStr">
@@ -575,13 +587,13 @@
           <t>September 16, 2026</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="2" t="n">
         <v>850</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="2" t="n">
         <v>918</v>
       </c>
       <c r="J3" t="inlineStr">
@@ -623,13 +635,13 @@
           <t>September 16, 2026</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="2" t="n">
         <v>850</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="2" t="n">
         <v>918</v>
       </c>
       <c r="J4" t="inlineStr">
@@ -641,6 +653,7 @@
       <c r="L4" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>